<commit_message>
text updated new results
</commit_message>
<xml_diff>
--- a/outputs/barcelona_samples_2015_2023_joined_results.xlsx
+++ b/outputs/barcelona_samples_2015_2023_joined_results.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="82">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t xml:space="preserve">bl_fin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">match</t>
   </si>
   <si>
     <t xml:space="preserve">usable</t>
@@ -275,7 +278,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -298,13 +301,26 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC9211E"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFD7"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -341,7 +357,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -350,11 +366,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -367,6 +399,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFD7"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FFC9211E"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -550,7 +642,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:O42"/>
+  <dimension ref="A2:P41"/>
   <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -599,95 +691,103 @@
       <c r="O2" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="P2" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="3" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L3),ISBLANK(M3)),"",IF(B3="ADD",AND(L3=1,M3=0),IF(B3="REMOVE",AND(L3=0,M3=1),IF(B3="NONCI",AND(L3=0,M3=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O3" s="1" t="n">
+        <f aca="false">IF(AND(NOT(ISBLANK(L3)),NOT(ISBLANK(M3))),1,"")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="L3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="1" t="n">
-        <f aca="false">IF(AND(NOT(ISBLANK(L3)),NOT(ISBLANK(M3))),1,"")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="L4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" s="1" t="n">
+      <c r="E4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L4),ISBLANK(M4)),"",IF(B4="ADD",AND(L4=1,M4=0),IF(B4="REMOVE",AND(L4=0,M4=1),IF(B4="NONCI",AND(L4=0,M4=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L4)),NOT(ISBLANK(M4))),1,"")</f>
         <v>1</v>
       </c>
@@ -697,13 +797,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>1</v>
@@ -723,7 +823,7 @@
       <c r="J5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="2" t="b">
+      <c r="K5" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -733,7 +833,11 @@
       <c r="M5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="1" t="n">
+      <c r="N5" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L5),ISBLANK(M5)),"",IF(B5="ADD",AND(L5=1,M5=0),IF(B5="REMOVE",AND(L5=0,M5=1),IF(B5="NONCI",AND(L5=0,M5=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O5" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L5)),NOT(ISBLANK(M5))),1,"")</f>
         <v>1</v>
       </c>
@@ -743,13 +847,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>1</v>
@@ -769,7 +873,7 @@
       <c r="J6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="2" t="b">
+      <c r="K6" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -779,7 +883,11 @@
       <c r="M6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N6" s="1" t="n">
+      <c r="N6" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L6),ISBLANK(M6)),"",IF(B6="ADD",AND(L6=1,M6=0),IF(B6="REMOVE",AND(L6=0,M6=1),IF(B6="NONCI",AND(L6=0,M6=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O6" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L6)),NOT(ISBLANK(M6))),1,"")</f>
         <v>1</v>
       </c>
@@ -789,13 +897,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>1</v>
@@ -815,7 +923,7 @@
       <c r="J7" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="2" t="b">
+      <c r="K7" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -825,7 +933,11 @@
       <c r="M7" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N7" s="1" t="n">
+      <c r="N7" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L7),ISBLANK(M7)),"",IF(B7="ADD",AND(L7=1,M7=0),IF(B7="REMOVE",AND(L7=0,M7=1),IF(B7="NONCI",AND(L7=0,M7=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O7" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L7)),NOT(ISBLANK(M7))),1,"")</f>
         <v>1</v>
       </c>
@@ -835,13 +947,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1</v>
@@ -861,7 +973,7 @@
       <c r="J8" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="2" t="b">
+      <c r="K8" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -871,7 +983,11 @@
       <c r="M8" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N8" s="1" t="n">
+      <c r="N8" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L8),ISBLANK(M8)),"",IF(B8="ADD",AND(L8=1,M8=0),IF(B8="REMOVE",AND(L8=0,M8=1),IF(B8="NONCI",AND(L8=0,M8=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O8" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L8)),NOT(ISBLANK(M8))),1,"")</f>
         <v>1</v>
       </c>
@@ -881,20 +997,17 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="E9" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="1" t="n">
-        <v>1</v>
-      </c>
       <c r="G9" s="1" t="n">
         <v>1</v>
       </c>
@@ -904,22 +1017,20 @@
       <c r="I9" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K9" s="3" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="L9" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="M9" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N9" s="1" t="n">
+      <c r="N9" s="1" t="str">
+        <f aca="false">IF(OR(ISBLANK(L9),ISBLANK(M9)),"",IF(B9="ADD",AND(L9=1,M9=0),IF(B9="REMOVE",AND(L9=0,M9=1),IF(B9="NONCI",AND(L9=0,M9=0),"" ))))</f>
+        <v/>
+      </c>
+      <c r="O9" s="1" t="str">
         <f aca="false">IF(AND(NOT(ISBLANK(L9)),NOT(ISBLANK(M9))),1,"")</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -927,19 +1038,38 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="K10" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="3" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="L10" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="N10" s="1" t="str">
+        <f aca="false">IF(OR(ISBLANK(L10),ISBLANK(M10)),"",IF(B10="ADD",AND(L10=1,M10=0),IF(B10="REMOVE",AND(L10=0,M10=1),IF(B10="NONCI",AND(L10=0,M10=0),"" ))))</f>
+        <v/>
+      </c>
+      <c r="O10" s="1" t="str">
         <f aca="false">IF(AND(NOT(ISBLANK(L10)),NOT(ISBLANK(M10))),1,"")</f>
         <v/>
       </c>
@@ -949,13 +1079,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>1</v>
@@ -975,7 +1105,7 @@
       <c r="J11" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="2" t="b">
+      <c r="K11" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -985,53 +1115,61 @@
       <c r="M11" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N11" s="1" t="n">
+      <c r="N11" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L11),ISBLANK(M11)),"",IF(B11="ADD",AND(L11=1,M11=0),IF(B11="REMOVE",AND(L11=0,M11=1),IF(B11="NONCI",AND(L11=0,M11=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O11" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L11)),NOT(ISBLANK(M11))),1,"")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="n">
+    <row r="12" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E12" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="L12" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="M12" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N12" s="1" t="n">
+      <c r="B12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L12),ISBLANK(M12)),"",IF(B12="ADD",AND(L12=1,M12=0),IF(B12="REMOVE",AND(L12=0,M12=1),IF(B12="NONCI",AND(L12=0,M12=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O12" s="4" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L12)),NOT(ISBLANK(M12))),1,"")</f>
         <v>1</v>
       </c>
@@ -1041,13 +1179,13 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>1</v>
@@ -1067,7 +1205,7 @@
       <c r="J13" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="2" t="b">
+      <c r="K13" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1077,7 +1215,11 @@
       <c r="M13" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N13" s="1" t="n">
+      <c r="N13" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L13),ISBLANK(M13)),"",IF(B13="ADD",AND(L13=1,M13=0),IF(B13="REMOVE",AND(L13=0,M13=1),IF(B13="NONCI",AND(L13=0,M13=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O13" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L13)),NOT(ISBLANK(M13))),1,"")</f>
         <v>1</v>
       </c>
@@ -1087,13 +1229,13 @@
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>1</v>
@@ -1113,7 +1255,7 @@
       <c r="J14" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="2" t="b">
+      <c r="K14" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1123,7 +1265,11 @@
       <c r="M14" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N14" s="1" t="n">
+      <c r="N14" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L14),ISBLANK(M14)),"",IF(B14="ADD",AND(L14=1,M14=0),IF(B14="REMOVE",AND(L14=0,M14=1),IF(B14="NONCI",AND(L14=0,M14=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O14" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L14)),NOT(ISBLANK(M14))),1,"")</f>
         <v>1</v>
       </c>
@@ -1133,13 +1279,13 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>1</v>
@@ -1159,7 +1305,7 @@
       <c r="J15" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="2" t="b">
+      <c r="K15" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1169,7 +1315,11 @@
       <c r="M15" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N15" s="1" t="n">
+      <c r="N15" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L15),ISBLANK(M15)),"",IF(B15="ADD",AND(L15=1,M15=0),IF(B15="REMOVE",AND(L15=0,M15=1),IF(B15="NONCI",AND(L15=0,M15=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O15" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L15)),NOT(ISBLANK(M15))),1,"")</f>
         <v>1</v>
       </c>
@@ -1179,13 +1329,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>1</v>
@@ -1205,7 +1355,7 @@
       <c r="J16" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="2" t="b">
+      <c r="K16" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1215,7 +1365,11 @@
       <c r="M16" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N16" s="1" t="n">
+      <c r="N16" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L16),ISBLANK(M16)),"",IF(B16="ADD",AND(L16=1,M16=0),IF(B16="REMOVE",AND(L16=0,M16=1),IF(B16="NONCI",AND(L16=0,M16=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O16" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L16)),NOT(ISBLANK(M16))),1,"")</f>
         <v>1</v>
       </c>
@@ -1225,14 +1379,14 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="E17" s="1" t="n">
         <v>1</v>
       </c>
@@ -1251,7 +1405,7 @@
       <c r="J17" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="2" t="b">
+      <c r="K17" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1261,47 +1415,61 @@
       <c r="M17" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N17" s="1" t="n">
+      <c r="N17" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L17),ISBLANK(M17)),"",IF(B17="ADD",AND(L17=1,M17=0),IF(B17="REMOVE",AND(L17=0,M17=1),IF(B17="NONCI",AND(L17=0,M17=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O17" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L17)),NOT(ISBLANK(M17))),1,"")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="n">
+    <row r="18" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C18" s="1" t="s">
+      <c r="B18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" s="2" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="L18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="1" t="n">
+      <c r="E18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L18),ISBLANK(M18)),"",IF(B18="ADD",AND(L18=1,M18=0),IF(B18="REMOVE",AND(L18=0,M18=1),IF(B18="NONCI",AND(L18=0,M18=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O18" s="4" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L18)),NOT(ISBLANK(M18))),1,"")</f>
         <v>1</v>
       </c>
@@ -1311,13 +1479,13 @@
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>1</v>
@@ -1337,7 +1505,7 @@
       <c r="J19" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="2" t="b">
+      <c r="K19" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1347,7 +1515,11 @@
       <c r="M19" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N19" s="1" t="n">
+      <c r="N19" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L19),ISBLANK(M19)),"",IF(B19="ADD",AND(L19=1,M19=0),IF(B19="REMOVE",AND(L19=0,M19=1),IF(B19="NONCI",AND(L19=0,M19=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O19" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L19)),NOT(ISBLANK(M19))),1,"")</f>
         <v>1</v>
       </c>
@@ -1357,13 +1529,13 @@
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>1</v>
@@ -1383,7 +1555,7 @@
       <c r="J20" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="2" t="b">
+      <c r="K20" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1393,93 +1565,105 @@
       <c r="M20" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N20" s="1" t="n">
+      <c r="N20" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L20),ISBLANK(M20)),"",IF(B20="ADD",AND(L20=1,M20=0),IF(B20="REMOVE",AND(L20=0,M20=1),IF(B20="NONCI",AND(L20=0,M20=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O20" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L20)),NOT(ISBLANK(M20))),1,"")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="n">
+    <row r="21" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D21" s="1" t="s">
+      <c r="B21" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E21" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" s="2" t="b">
+      <c r="D21" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L21" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="M21" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N21" s="1" t="n">
+      <c r="L21" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N21" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L21),ISBLANK(M21)),"",IF(B21="ADD",AND(L21=1,M21=0),IF(B21="REMOVE",AND(L21=0,M21=1),IF(B21="NONCI",AND(L21=0,M21=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O21" s="4" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L21)),NOT(ISBLANK(M21))),1,"")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="n">
+    <row r="22" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="1" t="s">
+      <c r="B22" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E22" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I22" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K22" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="L22" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="M22" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N22" s="1" t="n">
+      <c r="E22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L22),ISBLANK(M22)),"",IF(B22="ADD",AND(L22=1,M22=0),IF(B22="REMOVE",AND(L22=0,M22=1),IF(B22="NONCI",AND(L22=0,M22=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O22" s="4" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L22)),NOT(ISBLANK(M22))),1,"")</f>
         <v>1</v>
       </c>
@@ -1489,13 +1673,13 @@
         <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E23" s="1" t="n">
         <v>1</v>
@@ -1515,7 +1699,7 @@
       <c r="J23" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="2" t="b">
+      <c r="K23" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1525,7 +1709,11 @@
       <c r="M23" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N23" s="1" t="n">
+      <c r="N23" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L23),ISBLANK(M23)),"",IF(B23="ADD",AND(L23=1,M23=0),IF(B23="REMOVE",AND(L23=0,M23=1),IF(B23="NONCI",AND(L23=0,M23=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O23" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L23)),NOT(ISBLANK(M23))),1,"")</f>
         <v>1</v>
       </c>
@@ -1535,13 +1723,13 @@
         <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E24" s="1" t="n">
         <v>1</v>
@@ -1561,7 +1749,7 @@
       <c r="J24" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K24" s="2" t="b">
+      <c r="K24" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1571,7 +1759,11 @@
       <c r="M24" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N24" s="1" t="n">
+      <c r="N24" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L24),ISBLANK(M24)),"",IF(B24="ADD",AND(L24=1,M24=0),IF(B24="REMOVE",AND(L24=0,M24=1),IF(B24="NONCI",AND(L24=0,M24=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O24" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L24)),NOT(ISBLANK(M24))),1,"")</f>
         <v>1</v>
       </c>
@@ -1581,14 +1773,14 @@
         <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C25" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="E25" s="1" t="n">
         <v>1</v>
       </c>
@@ -1607,7 +1799,7 @@
       <c r="J25" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K25" s="2" t="b">
+      <c r="K25" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1617,7 +1809,11 @@
       <c r="M25" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N25" s="1" t="n">
+      <c r="N25" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L25),ISBLANK(M25)),"",IF(B25="ADD",AND(L25=1,M25=0),IF(B25="REMOVE",AND(L25=0,M25=1),IF(B25="NONCI",AND(L25=0,M25=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O25" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L25)),NOT(ISBLANK(M25))),1,"")</f>
         <v>1</v>
       </c>
@@ -1627,14 +1823,14 @@
         <v>24</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="E26" s="1" t="n">
         <v>1</v>
       </c>
@@ -1653,7 +1849,7 @@
       <c r="J26" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K26" s="2" t="b">
+      <c r="K26" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1663,7 +1859,11 @@
       <c r="M26" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N26" s="1" t="n">
+      <c r="N26" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L26),ISBLANK(M26)),"",IF(B26="ADD",AND(L26=1,M26=0),IF(B26="REMOVE",AND(L26=0,M26=1),IF(B26="NONCI",AND(L26=0,M26=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O26" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L26)),NOT(ISBLANK(M26))),1,"")</f>
         <v>1</v>
       </c>
@@ -1673,13 +1873,13 @@
         <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E27" s="1" t="n">
         <v>1</v>
@@ -1699,7 +1899,7 @@
       <c r="J27" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K27" s="2" t="b">
+      <c r="K27" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1709,7 +1909,11 @@
       <c r="M27" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N27" s="1" t="n">
+      <c r="N27" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L27),ISBLANK(M27)),"",IF(B27="ADD",AND(L27=1,M27=0),IF(B27="REMOVE",AND(L27=0,M27=1),IF(B27="NONCI",AND(L27=0,M27=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O27" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L27)),NOT(ISBLANK(M27))),1,"")</f>
         <v>1</v>
       </c>
@@ -1719,13 +1923,13 @@
         <v>26</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E28" s="1" t="n">
         <v>1</v>
@@ -1745,7 +1949,7 @@
       <c r="J28" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K28" s="2" t="b">
+      <c r="K28" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1755,7 +1959,11 @@
       <c r="M28" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N28" s="1" t="n">
+      <c r="N28" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L28),ISBLANK(M28)),"",IF(B28="ADD",AND(L28=1,M28=0),IF(B28="REMOVE",AND(L28=0,M28=1),IF(B28="NONCI",AND(L28=0,M28=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O28" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L28)),NOT(ISBLANK(M28))),1,"")</f>
         <v>1</v>
       </c>
@@ -1765,19 +1973,38 @@
         <v>27</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C29" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D29" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="K29" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="E29" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" s="3" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="L29" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="N29" s="1" t="str">
+        <f aca="false">IF(OR(ISBLANK(L29),ISBLANK(M29)),"",IF(B29="ADD",AND(L29=1,M29=0),IF(B29="REMOVE",AND(L29=0,M29=1),IF(B29="NONCI",AND(L29=0,M29=0),"" ))))</f>
+        <v/>
+      </c>
+      <c r="O29" s="1" t="str">
         <f aca="false">IF(AND(NOT(ISBLANK(L29)),NOT(ISBLANK(M29))),1,"")</f>
         <v/>
       </c>
@@ -1787,13 +2014,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>1</v>
@@ -1813,7 +2040,7 @@
       <c r="J30" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K30" s="2" t="b">
+      <c r="K30" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1823,7 +2050,11 @@
       <c r="M30" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N30" s="1" t="n">
+      <c r="N30" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L30),ISBLANK(M30)),"",IF(B30="ADD",AND(L30=1,M30=0),IF(B30="REMOVE",AND(L30=0,M30=1),IF(B30="NONCI",AND(L30=0,M30=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O30" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L30)),NOT(ISBLANK(M30))),1,"")</f>
         <v>1</v>
       </c>
@@ -1833,13 +2064,13 @@
         <v>29</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E31" s="1" t="n">
         <v>1</v>
@@ -1859,7 +2090,7 @@
       <c r="J31" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K31" s="2" t="b">
+      <c r="K31" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1869,7 +2100,11 @@
       <c r="M31" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N31" s="1" t="n">
+      <c r="N31" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L31),ISBLANK(M31)),"",IF(B31="ADD",AND(L31=1,M31=0),IF(B31="REMOVE",AND(L31=0,M31=1),IF(B31="NONCI",AND(L31=0,M31=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O31" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L31)),NOT(ISBLANK(M31))),1,"")</f>
         <v>1</v>
       </c>
@@ -1879,13 +2114,13 @@
         <v>30</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E32" s="1" t="n">
         <v>1</v>
@@ -1905,7 +2140,7 @@
       <c r="J32" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K32" s="2" t="b">
+      <c r="K32" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1915,7 +2150,11 @@
       <c r="M32" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N32" s="1" t="n">
+      <c r="N32" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L32),ISBLANK(M32)),"",IF(B32="ADD",AND(L32=1,M32=0),IF(B32="REMOVE",AND(L32=0,M32=1),IF(B32="NONCI",AND(L32=0,M32=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O32" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L32)),NOT(ISBLANK(M32))),1,"")</f>
         <v>1</v>
       </c>
@@ -1925,19 +2164,38 @@
         <v>31</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="K33" s="2" t="b">
-        <f aca="false">FALSE()</f>
+        <v>45</v>
+      </c>
+      <c r="F33" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="3" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="M33" s="1" t="n">
         <v>0</v>
       </c>
       <c r="N33" s="1" t="str">
+        <f aca="false">IF(OR(ISBLANK(L33),ISBLANK(M33)),"",IF(B33="ADD",AND(L33=1,M33=0),IF(B33="REMOVE",AND(L33=0,M33=1),IF(B33="NONCI",AND(L33=0,M33=0),"" ))))</f>
+        <v/>
+      </c>
+      <c r="O33" s="1" t="str">
         <f aca="false">IF(AND(NOT(ISBLANK(L33)),NOT(ISBLANK(M33))),1,"")</f>
         <v/>
       </c>
@@ -1947,14 +2205,14 @@
         <v>32</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C34" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D34" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="E34" s="1" t="n">
         <v>1</v>
       </c>
@@ -1973,7 +2231,7 @@
       <c r="J34" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K34" s="2" t="b">
+      <c r="K34" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1983,7 +2241,11 @@
       <c r="M34" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N34" s="1" t="n">
+      <c r="N34" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L34),ISBLANK(M34)),"",IF(B34="ADD",AND(L34=1,M34=0),IF(B34="REMOVE",AND(L34=0,M34=1),IF(B34="NONCI",AND(L34=0,M34=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O34" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L34)),NOT(ISBLANK(M34))),1,"")</f>
         <v>1</v>
       </c>
@@ -1993,20 +2255,17 @@
         <v>33</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C35" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D35" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="E35" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F35" s="1" t="n">
-        <v>1</v>
-      </c>
       <c r="G35" s="1" t="n">
         <v>1</v>
       </c>
@@ -2016,22 +2275,20 @@
       <c r="I35" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="J35" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K35" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="K35" s="3" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="L35" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="M35" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N35" s="1" t="n">
+      <c r="N35" s="1" t="str">
+        <f aca="false">IF(OR(ISBLANK(L35),ISBLANK(M35)),"",IF(B35="ADD",AND(L35=1,M35=0),IF(B35="REMOVE",AND(L35=0,M35=1),IF(B35="NONCI",AND(L35=0,M35=0),"" ))))</f>
+        <v/>
+      </c>
+      <c r="O35" s="1" t="str">
         <f aca="false">IF(AND(NOT(ISBLANK(L35)),NOT(ISBLANK(M35))),1,"")</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2039,13 +2296,13 @@
         <v>34</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E36" s="1" t="n">
         <v>1</v>
@@ -2065,7 +2322,7 @@
       <c r="J36" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K36" s="2" t="b">
+      <c r="K36" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -2075,7 +2332,11 @@
       <c r="M36" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N36" s="1" t="n">
+      <c r="N36" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L36),ISBLANK(M36)),"",IF(B36="ADD",AND(L36=1,M36=0),IF(B36="REMOVE",AND(L36=0,M36=1),IF(B36="NONCI",AND(L36=0,M36=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O36" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L36)),NOT(ISBLANK(M36))),1,"")</f>
         <v>1</v>
       </c>
@@ -2085,13 +2346,13 @@
         <v>35</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E37" s="1" t="n">
         <v>1</v>
@@ -2111,7 +2372,7 @@
       <c r="J37" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K37" s="2" t="b">
+      <c r="K37" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -2121,7 +2382,11 @@
       <c r="M37" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N37" s="1" t="n">
+      <c r="N37" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L37),ISBLANK(M37)),"",IF(B37="ADD",AND(L37=1,M37=0),IF(B37="REMOVE",AND(L37=0,M37=1),IF(B37="NONCI",AND(L37=0,M37=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O37" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L37)),NOT(ISBLANK(M37))),1,"")</f>
         <v>1</v>
       </c>
@@ -2131,14 +2396,14 @@
         <v>36</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C38" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D38" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="E38" s="1" t="n">
         <v>1</v>
       </c>
@@ -2157,7 +2422,7 @@
       <c r="J38" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K38" s="2" t="b">
+      <c r="K38" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -2167,7 +2432,11 @@
       <c r="M38" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N38" s="1" t="n">
+      <c r="N38" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L38),ISBLANK(M38)),"",IF(B38="ADD",AND(L38=1,M38=0),IF(B38="REMOVE",AND(L38=0,M38=1),IF(B38="NONCI",AND(L38=0,M38=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O38" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L38)),NOT(ISBLANK(M38))),1,"")</f>
         <v>1</v>
       </c>
@@ -2177,19 +2446,38 @@
         <v>37</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="K39" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>49</v>
+      </c>
+      <c r="E39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" s="3" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="L39" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="N39" s="1" t="str">
+        <f aca="false">IF(OR(ISBLANK(L39),ISBLANK(M39)),"",IF(B39="ADD",AND(L39=1,M39=0),IF(B39="REMOVE",AND(L39=0,M39=1),IF(B39="NONCI",AND(L39=0,M39=0),"" ))))</f>
+        <v/>
+      </c>
+      <c r="O39" s="1" t="str">
         <f aca="false">IF(AND(NOT(ISBLANK(L39)),NOT(ISBLANK(M39))),1,"")</f>
         <v/>
       </c>
@@ -2199,13 +2487,13 @@
         <v>38</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E40" s="1" t="n">
         <v>1</v>
@@ -2213,8 +2501,8 @@
       <c r="F40" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G40" s="1" t="n">
-        <v>0</v>
+      <c r="G40" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="H40" s="1" t="n">
         <v>0</v>
@@ -2222,75 +2510,73 @@
       <c r="J40" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K40" s="2" t="b">
+      <c r="K40" s="3" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L40" s="1" t="n">
+      <c r="L40" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M40" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N40" s="1" t="n">
+      <c r="N40" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L40),ISBLANK(M40)),"",IF(B40="ADD",AND(L40=1,M40=0),IF(B40="REMOVE",AND(L40=0,M40=1),IF(B40="NONCI",AND(L40=0,M40=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O40" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L40)),NOT(ISBLANK(M40))),1,"")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="1" t="n">
+    <row r="41" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="B41" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K41" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="L41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N41" s="1" t="n">
+      <c r="B41" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L41),ISBLANK(M41)),"",IF(B41="ADD",AND(L41=1,M41=0),IF(B41="REMOVE",AND(L41=0,M41=1),IF(B41="NONCI",AND(L41=0,M41=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O41" s="4" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L41)),NOT(ISBLANK(M41))),1,"")</f>
         <v>1</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K42" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="N42" s="1" t="str">
-        <f aca="false">IF(AND(NOT(ISBLANK(L42)),NOT(ISBLANK(M42))),1,"")</f>
-        <v/>
       </c>
     </row>
   </sheetData>
@@ -2309,7 +2595,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:O8"/>
+  <dimension ref="A2:P8"/>
   <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2358,135 +2644,150 @@
       <c r="O2" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="P2" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="L3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="1" t="n">
+      <c r="D3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L3),ISBLANK(M3)),"",IF(B3="ADD",AND(L3=1,M3=0),IF(B3="REMOVE",AND(L3=0,M3=1),IF(B3="NONCI",AND(L3=0,M3=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O3" s="4" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L3)),NOT(ISBLANK(M3))),1,"")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
+    <row r="4" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="B4" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="C4" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L4),ISBLANK(M4)),"",IF(B4="ADD",AND(L4=1,M4=0),IF(B4="REMOVE",AND(L4=0,M4=1),IF(B4="NONCI",AND(L4=0,M4=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <f aca="false">IF(AND(NOT(ISBLANK(L4)),NOT(ISBLANK(M4))),1,"")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="L4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="1" t="n">
-        <f aca="false">IF(AND(NOT(ISBLANK(L4)),NOT(ISBLANK(M4))),1,"")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" s="2" t="b">
+      <c r="D5" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="1" t="n">
+      <c r="L5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L5),ISBLANK(M5)),"",IF(B5="ADD",AND(L5=1,M5=0),IF(B5="REMOVE",AND(L5=0,M5=1),IF(B5="NONCI",AND(L5=0,M5=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O5" s="4" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L5)),NOT(ISBLANK(M5))),1,"")</f>
         <v>1</v>
       </c>
@@ -2496,14 +2797,14 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>38</v>
-      </c>
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
@@ -2522,7 +2823,7 @@
       <c r="J6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="K6" s="2" t="b">
+      <c r="K6" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -2532,7 +2833,11 @@
       <c r="M6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="N6" s="1" t="n">
+      <c r="N6" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L6),ISBLANK(M6)),"",IF(B6="ADD",AND(L6=1,M6=0),IF(B6="REMOVE",AND(L6=0,M6=1),IF(B6="NONCI",AND(L6=0,M6=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O6" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L6)),NOT(ISBLANK(M6))),1,"")</f>
         <v>1</v>
       </c>
@@ -2542,65 +2847,88 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="K7" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="E7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="3" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="L7" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="N7" s="1" t="str">
+        <f aca="false">IF(OR(ISBLANK(L7),ISBLANK(M7)),"",IF(B7="ADD",AND(L7=1,M7=0),IF(B7="REMOVE",AND(L7=0,M7=1),IF(B7="NONCI",AND(L7=0,M7=0),"" ))))</f>
+        <v/>
+      </c>
+      <c r="O7" s="1" t="str">
         <f aca="false">IF(AND(NOT(ISBLANK(L7)),NOT(ISBLANK(M7))),1,"")</f>
         <v/>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="n">
+    <row r="8" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="L8" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="1" t="n">
+      <c r="B8" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L8),ISBLANK(M8)),"",IF(B8="ADD",AND(L8=1,M8=0),IF(B8="REMOVE",AND(L8=0,M8=1),IF(B8="NONCI",AND(L8=0,M8=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O8" s="4" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L8)),NOT(ISBLANK(M8))),1,"")</f>
         <v>1</v>
       </c>
@@ -2621,7 +2949,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:O52"/>
+  <dimension ref="A2:P52"/>
   <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2670,19 +2998,22 @@
       <c r="O2" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="P2" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>0</v>
@@ -2702,7 +3033,7 @@
       <c r="J3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K3" s="2" t="b">
+      <c r="K3" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -2712,7 +3043,11 @@
       <c r="M3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N3" s="1" t="n">
+      <c r="N3" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L3),ISBLANK(M3)),"",IF(B3="ADD",AND(L3=1,M3=0),IF(B3="REMOVE",AND(L3=0,M3=1),IF(B3="NONCI",AND(L3=0,M3=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O3" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L3)),NOT(ISBLANK(M3))),1,"")</f>
         <v>1</v>
       </c>
@@ -2722,13 +3057,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
@@ -2748,7 +3083,7 @@
       <c r="J4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K4" s="2" t="b">
+      <c r="K4" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -2758,7 +3093,11 @@
       <c r="M4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N4" s="1" t="n">
+      <c r="N4" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L4),ISBLANK(M4)),"",IF(B4="ADD",AND(L4=1,M4=0),IF(B4="REMOVE",AND(L4=0,M4=1),IF(B4="NONCI",AND(L4=0,M4=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O4" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L4)),NOT(ISBLANK(M4))),1,"")</f>
         <v>1</v>
       </c>
@@ -2768,14 +3107,14 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
@@ -2794,7 +3133,7 @@
       <c r="J5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="2" t="b">
+      <c r="K5" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -2804,50 +3143,58 @@
       <c r="M5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="1" t="n">
+      <c r="N5" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L5),ISBLANK(M5)),"",IF(B5="ADD",AND(L5=1,M5=0),IF(B5="REMOVE",AND(L5=0,M5=1),IF(B5="NONCI",AND(L5=0,M5=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O5" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L5)),NOT(ISBLANK(M5))),1,"")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
+    <row r="6" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="2" t="b">
+      <c r="B6" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="1" t="n">
+      <c r="L6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L6),ISBLANK(M6)),"",IF(B6="ADD",AND(L6=1,M6=0),IF(B6="REMOVE",AND(L6=0,M6=1),IF(B6="NONCI",AND(L6=0,M6=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L6)),NOT(ISBLANK(M6))),1,"")</f>
         <v>1</v>
       </c>
@@ -2857,13 +3204,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0</v>
@@ -2883,7 +3230,7 @@
       <c r="J7" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="2" t="b">
+      <c r="K7" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -2893,7 +3240,11 @@
       <c r="M7" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N7" s="1" t="n">
+      <c r="N7" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L7),ISBLANK(M7)),"",IF(B7="ADD",AND(L7=1,M7=0),IF(B7="REMOVE",AND(L7=0,M7=1),IF(B7="NONCI",AND(L7=0,M7=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O7" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L7)),NOT(ISBLANK(M7))),1,"")</f>
         <v>1</v>
       </c>
@@ -2903,13 +3254,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>0</v>
@@ -2929,7 +3280,7 @@
       <c r="J8" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="2" t="b">
+      <c r="K8" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -2939,7 +3290,11 @@
       <c r="M8" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N8" s="1" t="n">
+      <c r="N8" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L8),ISBLANK(M8)),"",IF(B8="ADD",AND(L8=1,M8=0),IF(B8="REMOVE",AND(L8=0,M8=1),IF(B8="NONCI",AND(L8=0,M8=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O8" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L8)),NOT(ISBLANK(M8))),1,"")</f>
         <v>1</v>
       </c>
@@ -2949,13 +3304,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
@@ -2975,7 +3330,7 @@
       <c r="J9" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="2" t="b">
+      <c r="K9" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -2985,7 +3340,11 @@
       <c r="M9" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N9" s="1" t="n">
+      <c r="N9" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L9),ISBLANK(M9)),"",IF(B9="ADD",AND(L9=1,M9=0),IF(B9="REMOVE",AND(L9=0,M9=1),IF(B9="NONCI",AND(L9=0,M9=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O9" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L9)),NOT(ISBLANK(M9))),1,"")</f>
         <v>1</v>
       </c>
@@ -2995,13 +3354,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
@@ -3021,7 +3380,7 @@
       <c r="J10" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="2" t="b">
+      <c r="K10" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3031,7 +3390,11 @@
       <c r="M10" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N10" s="1" t="n">
+      <c r="N10" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L10),ISBLANK(M10)),"",IF(B10="ADD",AND(L10=1,M10=0),IF(B10="REMOVE",AND(L10=0,M10=1),IF(B10="NONCI",AND(L10=0,M10=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O10" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L10)),NOT(ISBLANK(M10))),1,"")</f>
         <v>1</v>
       </c>
@@ -3041,14 +3404,14 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="F11" s="1" t="n">
         <v>0</v>
       </c>
@@ -3058,7 +3421,7 @@
       <c r="J11" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="2" t="b">
+      <c r="K11" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3066,6 +3429,10 @@
         <v>0</v>
       </c>
       <c r="N11" s="1" t="str">
+        <f aca="false">IF(OR(ISBLANK(L11),ISBLANK(M11)),"",IF(B11="ADD",AND(L11=1,M11=0),IF(B11="REMOVE",AND(L11=0,M11=1),IF(B11="NONCI",AND(L11=0,M11=0),"" ))))</f>
+        <v/>
+      </c>
+      <c r="O11" s="1" t="str">
         <f aca="false">IF(AND(NOT(ISBLANK(L11)),NOT(ISBLANK(M11))),1,"")</f>
         <v/>
       </c>
@@ -3075,19 +3442,23 @@
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="K12" s="2" t="b">
+        <v>23</v>
+      </c>
+      <c r="K12" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="N12" s="1" t="str">
+        <f aca="false">IF(OR(ISBLANK(L12),ISBLANK(M12)),"",IF(B12="ADD",AND(L12=1,M12=0),IF(B12="REMOVE",AND(L12=0,M12=1),IF(B12="NONCI",AND(L12=0,M12=0),"" ))))</f>
+        <v/>
+      </c>
+      <c r="O12" s="1" t="str">
         <f aca="false">IF(AND(NOT(ISBLANK(L12)),NOT(ISBLANK(M12))),1,"")</f>
         <v/>
       </c>
@@ -3097,13 +3468,13 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
@@ -3123,7 +3494,7 @@
       <c r="J13" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="2" t="b">
+      <c r="K13" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3133,7 +3504,11 @@
       <c r="M13" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N13" s="1" t="n">
+      <c r="N13" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L13),ISBLANK(M13)),"",IF(B13="ADD",AND(L13=1,M13=0),IF(B13="REMOVE",AND(L13=0,M13=1),IF(B13="NONCI",AND(L13=0,M13=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O13" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L13)),NOT(ISBLANK(M13))),1,"")</f>
         <v>1</v>
       </c>
@@ -3143,13 +3518,13 @@
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0</v>
@@ -3169,7 +3544,7 @@
       <c r="J14" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="2" t="b">
+      <c r="K14" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3179,7 +3554,11 @@
       <c r="M14" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N14" s="1" t="n">
+      <c r="N14" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L14),ISBLANK(M14)),"",IF(B14="ADD",AND(L14=1,M14=0),IF(B14="REMOVE",AND(L14=0,M14=1),IF(B14="NONCI",AND(L14=0,M14=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O14" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L14)),NOT(ISBLANK(M14))),1,"")</f>
         <v>1</v>
       </c>
@@ -3189,13 +3568,13 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0</v>
@@ -3215,7 +3594,7 @@
       <c r="J15" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="2" t="b">
+      <c r="K15" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3225,7 +3604,11 @@
       <c r="M15" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N15" s="1" t="n">
+      <c r="N15" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L15),ISBLANK(M15)),"",IF(B15="ADD",AND(L15=1,M15=0),IF(B15="REMOVE",AND(L15=0,M15=1),IF(B15="NONCI",AND(L15=0,M15=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O15" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L15)),NOT(ISBLANK(M15))),1,"")</f>
         <v>1</v>
       </c>
@@ -3235,13 +3618,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>0</v>
@@ -3261,7 +3644,7 @@
       <c r="J16" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="2" t="b">
+      <c r="K16" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3271,7 +3654,11 @@
       <c r="M16" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N16" s="1" t="n">
+      <c r="N16" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L16),ISBLANK(M16)),"",IF(B16="ADD",AND(L16=1,M16=0),IF(B16="REMOVE",AND(L16=0,M16=1),IF(B16="NONCI",AND(L16=0,M16=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O16" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L16)),NOT(ISBLANK(M16))),1,"")</f>
         <v>1</v>
       </c>
@@ -3281,13 +3668,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0</v>
@@ -3307,7 +3694,7 @@
       <c r="J17" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="2" t="b">
+      <c r="K17" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3317,53 +3704,61 @@
       <c r="M17" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N17" s="1" t="n">
+      <c r="N17" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L17),ISBLANK(M17)),"",IF(B17="ADD",AND(L17=1,M17=0),IF(B17="REMOVE",AND(L17=0,M17=1),IF(B17="NONCI",AND(L17=0,M17=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O17" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L17)),NOT(ISBLANK(M17))),1,"")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="n">
+    <row r="18" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I18" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="L18" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="M18" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N18" s="1" t="n">
+      <c r="B18" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L18),ISBLANK(M18)),"",IF(B18="ADD",AND(L18=1,M18=0),IF(B18="REMOVE",AND(L18=0,M18=1),IF(B18="NONCI",AND(L18=0,M18=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O18" s="4" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L18)),NOT(ISBLANK(M18))),1,"")</f>
         <v>1</v>
       </c>
@@ -3373,14 +3768,14 @@
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="E19" s="1" t="n">
         <v>0</v>
       </c>
@@ -3399,7 +3794,7 @@
       <c r="J19" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="2" t="b">
+      <c r="K19" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3409,7 +3804,11 @@
       <c r="M19" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N19" s="1" t="n">
+      <c r="N19" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L19),ISBLANK(M19)),"",IF(B19="ADD",AND(L19=1,M19=0),IF(B19="REMOVE",AND(L19=0,M19=1),IF(B19="NONCI",AND(L19=0,M19=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O19" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L19)),NOT(ISBLANK(M19))),1,"")</f>
         <v>1</v>
       </c>
@@ -3419,13 +3818,13 @@
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>0</v>
@@ -3445,7 +3844,7 @@
       <c r="J20" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="2" t="b">
+      <c r="K20" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3455,7 +3854,11 @@
       <c r="M20" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N20" s="1" t="n">
+      <c r="N20" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L20),ISBLANK(M20)),"",IF(B20="ADD",AND(L20=1,M20=0),IF(B20="REMOVE",AND(L20=0,M20=1),IF(B20="NONCI",AND(L20=0,M20=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O20" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L20)),NOT(ISBLANK(M20))),1,"")</f>
         <v>1</v>
       </c>
@@ -3465,13 +3868,13 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E21" s="1" t="n">
         <v>0</v>
@@ -3491,7 +3894,7 @@
       <c r="J21" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K21" s="2" t="b">
+      <c r="K21" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3501,7 +3904,11 @@
       <c r="M21" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N21" s="1" t="n">
+      <c r="N21" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L21),ISBLANK(M21)),"",IF(B21="ADD",AND(L21=1,M21=0),IF(B21="REMOVE",AND(L21=0,M21=1),IF(B21="NONCI",AND(L21=0,M21=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O21" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L21)),NOT(ISBLANK(M21))),1,"")</f>
         <v>1</v>
       </c>
@@ -3511,13 +3918,13 @@
         <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0</v>
@@ -3537,7 +3944,7 @@
       <c r="J22" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="2" t="b">
+      <c r="K22" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3547,7 +3954,11 @@
       <c r="M22" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N22" s="1" t="n">
+      <c r="N22" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L22),ISBLANK(M22)),"",IF(B22="ADD",AND(L22=1,M22=0),IF(B22="REMOVE",AND(L22=0,M22=1),IF(B22="NONCI",AND(L22=0,M22=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O22" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L22)),NOT(ISBLANK(M22))),1,"")</f>
         <v>1</v>
       </c>
@@ -3557,89 +3968,97 @@
         <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="3" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L23),ISBLANK(M23)),"",IF(B23="ADD",AND(L23=1,M23=0),IF(B23="REMOVE",AND(L23=0,M23=1),IF(B23="NONCI",AND(L23=0,M23=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O23" s="1" t="n">
+        <f aca="false">IF(AND(NOT(ISBLANK(L23)),NOT(ISBLANK(M23))),1,"")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="L23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="1" t="n">
-        <f aca="false">IF(AND(NOT(ISBLANK(L23)),NOT(ISBLANK(M23))),1,"")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K24" s="2" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="L24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="M24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N24" s="1" t="n">
+      <c r="D24" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" s="5" t="b">
+        <f aca="false">IF(OR(ISBLANK(L24),ISBLANK(M24)),"",IF(B24="ADD",AND(L24=1,M24=0),IF(B24="REMOVE",AND(L24=0,M24=1),IF(B24="NONCI",AND(L24=0,M24=0),"" ))))</f>
+        <v>0</v>
+      </c>
+      <c r="O24" s="4" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L24)),NOT(ISBLANK(M24))),1,"")</f>
         <v>1</v>
       </c>
@@ -3649,14 +4068,14 @@
         <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C25" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="E25" s="1" t="n">
         <v>0</v>
       </c>
@@ -3675,7 +4094,7 @@
       <c r="J25" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K25" s="2" t="b">
+      <c r="K25" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3685,7 +4104,11 @@
       <c r="M25" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N25" s="1" t="n">
+      <c r="N25" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L25),ISBLANK(M25)),"",IF(B25="ADD",AND(L25=1,M25=0),IF(B25="REMOVE",AND(L25=0,M25=1),IF(B25="NONCI",AND(L25=0,M25=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O25" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L25)),NOT(ISBLANK(M25))),1,"")</f>
         <v>1</v>
       </c>
@@ -3695,13 +4118,13 @@
         <v>24</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E26" s="1" t="n">
         <v>0</v>
@@ -3721,7 +4144,7 @@
       <c r="J26" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K26" s="2" t="b">
+      <c r="K26" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3731,7 +4154,11 @@
       <c r="M26" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N26" s="1" t="n">
+      <c r="N26" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L26),ISBLANK(M26)),"",IF(B26="ADD",AND(L26=1,M26=0),IF(B26="REMOVE",AND(L26=0,M26=1),IF(B26="NONCI",AND(L26=0,M26=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O26" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L26)),NOT(ISBLANK(M26))),1,"")</f>
         <v>1</v>
       </c>
@@ -3741,13 +4168,13 @@
         <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E27" s="1" t="n">
         <v>0</v>
@@ -3767,7 +4194,7 @@
       <c r="J27" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K27" s="2" t="b">
+      <c r="K27" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3777,7 +4204,11 @@
       <c r="M27" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N27" s="1" t="n">
+      <c r="N27" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L27),ISBLANK(M27)),"",IF(B27="ADD",AND(L27=1,M27=0),IF(B27="REMOVE",AND(L27=0,M27=1),IF(B27="NONCI",AND(L27=0,M27=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O27" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L27)),NOT(ISBLANK(M27))),1,"")</f>
         <v>1</v>
       </c>
@@ -3787,13 +4218,13 @@
         <v>26</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E28" s="1" t="n">
         <v>0</v>
@@ -3804,20 +4235,27 @@
       <c r="G28" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="H28" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I28" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K28" s="2" t="b">
+      <c r="K28" s="3" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="L28" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="M28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" s="1" t="n">
+      <c r="M28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L28),ISBLANK(M28)),"",IF(B28="ADD",AND(L28=1,M28=0),IF(B28="REMOVE",AND(L28=0,M28=1),IF(B28="NONCI",AND(L28=0,M28=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O28" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L28)),NOT(ISBLANK(M28))),1,"")</f>
         <v>1</v>
       </c>
@@ -3827,13 +4265,13 @@
         <v>27</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E29" s="1" t="n">
         <v>0</v>
@@ -3853,7 +4291,7 @@
       <c r="J29" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K29" s="2" t="b">
+      <c r="K29" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3863,7 +4301,11 @@
       <c r="M29" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N29" s="1" t="n">
+      <c r="N29" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L29),ISBLANK(M29)),"",IF(B29="ADD",AND(L29=1,M29=0),IF(B29="REMOVE",AND(L29=0,M29=1),IF(B29="NONCI",AND(L29=0,M29=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O29" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L29)),NOT(ISBLANK(M29))),1,"")</f>
         <v>1</v>
       </c>
@@ -3873,13 +4315,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>0</v>
@@ -3887,23 +4329,30 @@
       <c r="F30" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="G30" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="H30" s="1" t="n">
         <v>0</v>
       </c>
       <c r="J30" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K30" s="2" t="b">
+      <c r="K30" s="3" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="L30" s="0" t="n">
+      <c r="L30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M30" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N30" s="1" t="n">
+      <c r="N30" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L30),ISBLANK(M30)),"",IF(B30="ADD",AND(L30=1,M30=0),IF(B30="REMOVE",AND(L30=0,M30=1),IF(B30="NONCI",AND(L30=0,M30=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O30" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L30)),NOT(ISBLANK(M30))),1,"")</f>
         <v>1</v>
       </c>
@@ -3913,14 +4362,14 @@
         <v>29</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C31" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D31" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="E31" s="1" t="n">
         <v>0</v>
       </c>
@@ -3939,7 +4388,7 @@
       <c r="J31" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K31" s="2" t="b">
+      <c r="K31" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3949,7 +4398,11 @@
       <c r="M31" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N31" s="1" t="n">
+      <c r="N31" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L31),ISBLANK(M31)),"",IF(B31="ADD",AND(L31=1,M31=0),IF(B31="REMOVE",AND(L31=0,M31=1),IF(B31="NONCI",AND(L31=0,M31=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O31" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L31)),NOT(ISBLANK(M31))),1,"")</f>
         <v>1</v>
       </c>
@@ -3959,13 +4412,13 @@
         <v>30</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E32" s="1" t="n">
         <v>0</v>
@@ -3985,7 +4438,7 @@
       <c r="J32" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K32" s="2" t="b">
+      <c r="K32" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -3995,7 +4448,11 @@
       <c r="M32" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N32" s="1" t="n">
+      <c r="N32" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L32),ISBLANK(M32)),"",IF(B32="ADD",AND(L32=1,M32=0),IF(B32="REMOVE",AND(L32=0,M32=1),IF(B32="NONCI",AND(L32=0,M32=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O32" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L32)),NOT(ISBLANK(M32))),1,"")</f>
         <v>1</v>
       </c>
@@ -4005,13 +4462,13 @@
         <v>31</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E33" s="1" t="n">
         <v>0</v>
@@ -4031,7 +4488,7 @@
       <c r="J33" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K33" s="2" t="b">
+      <c r="K33" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4041,7 +4498,11 @@
       <c r="M33" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N33" s="1" t="n">
+      <c r="N33" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L33),ISBLANK(M33)),"",IF(B33="ADD",AND(L33=1,M33=0),IF(B33="REMOVE",AND(L33=0,M33=1),IF(B33="NONCI",AND(L33=0,M33=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O33" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L33)),NOT(ISBLANK(M33))),1,"")</f>
         <v>1</v>
       </c>
@@ -4051,13 +4512,13 @@
         <v>32</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E34" s="1" t="n">
         <v>0</v>
@@ -4077,7 +4538,7 @@
       <c r="J34" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K34" s="2" t="b">
+      <c r="K34" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4087,7 +4548,11 @@
       <c r="M34" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N34" s="1" t="n">
+      <c r="N34" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L34),ISBLANK(M34)),"",IF(B34="ADD",AND(L34=1,M34=0),IF(B34="REMOVE",AND(L34=0,M34=1),IF(B34="NONCI",AND(L34=0,M34=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O34" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L34)),NOT(ISBLANK(M34))),1,"")</f>
         <v>1</v>
       </c>
@@ -4097,13 +4562,13 @@
         <v>33</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E35" s="1" t="n">
         <v>0</v>
@@ -4123,7 +4588,7 @@
       <c r="J35" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K35" s="2" t="b">
+      <c r="K35" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4133,7 +4598,11 @@
       <c r="M35" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N35" s="1" t="n">
+      <c r="N35" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L35),ISBLANK(M35)),"",IF(B35="ADD",AND(L35=1,M35=0),IF(B35="REMOVE",AND(L35=0,M35=1),IF(B35="NONCI",AND(L35=0,M35=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O35" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L35)),NOT(ISBLANK(M35))),1,"")</f>
         <v>1</v>
       </c>
@@ -4143,13 +4612,13 @@
         <v>34</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E36" s="1" t="n">
         <v>0</v>
@@ -4169,7 +4638,7 @@
       <c r="J36" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K36" s="2" t="b">
+      <c r="K36" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4179,7 +4648,11 @@
       <c r="M36" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N36" s="1" t="n">
+      <c r="N36" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L36),ISBLANK(M36)),"",IF(B36="ADD",AND(L36=1,M36=0),IF(B36="REMOVE",AND(L36=0,M36=1),IF(B36="NONCI",AND(L36=0,M36=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O36" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L36)),NOT(ISBLANK(M36))),1,"")</f>
         <v>1</v>
       </c>
@@ -4189,13 +4662,13 @@
         <v>35</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E37" s="1" t="n">
         <v>0</v>
@@ -4215,7 +4688,7 @@
       <c r="J37" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K37" s="2" t="b">
+      <c r="K37" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4225,7 +4698,11 @@
       <c r="M37" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N37" s="1" t="n">
+      <c r="N37" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L37),ISBLANK(M37)),"",IF(B37="ADD",AND(L37=1,M37=0),IF(B37="REMOVE",AND(L37=0,M37=1),IF(B37="NONCI",AND(L37=0,M37=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O37" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L37)),NOT(ISBLANK(M37))),1,"")</f>
         <v>1</v>
       </c>
@@ -4235,13 +4712,13 @@
         <v>36</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E38" s="1" t="n">
         <v>0</v>
@@ -4261,7 +4738,7 @@
       <c r="J38" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K38" s="2" t="b">
+      <c r="K38" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4271,7 +4748,11 @@
       <c r="M38" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N38" s="1" t="n">
+      <c r="N38" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L38),ISBLANK(M38)),"",IF(B38="ADD",AND(L38=1,M38=0),IF(B38="REMOVE",AND(L38=0,M38=1),IF(B38="NONCI",AND(L38=0,M38=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O38" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L38)),NOT(ISBLANK(M38))),1,"")</f>
         <v>1</v>
       </c>
@@ -4281,13 +4762,13 @@
         <v>37</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E39" s="1" t="n">
         <v>0</v>
@@ -4307,7 +4788,7 @@
       <c r="J39" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K39" s="2" t="b">
+      <c r="K39" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4317,7 +4798,11 @@
       <c r="M39" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N39" s="1" t="n">
+      <c r="N39" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L39),ISBLANK(M39)),"",IF(B39="ADD",AND(L39=1,M39=0),IF(B39="REMOVE",AND(L39=0,M39=1),IF(B39="NONCI",AND(L39=0,M39=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O39" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L39)),NOT(ISBLANK(M39))),1,"")</f>
         <v>1</v>
       </c>
@@ -4327,13 +4812,13 @@
         <v>38</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E40" s="1" t="n">
         <v>0</v>
@@ -4353,7 +4838,7 @@
       <c r="J40" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K40" s="2" t="b">
+      <c r="K40" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4363,7 +4848,11 @@
       <c r="M40" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N40" s="1" t="n">
+      <c r="N40" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L40),ISBLANK(M40)),"",IF(B40="ADD",AND(L40=1,M40=0),IF(B40="REMOVE",AND(L40=0,M40=1),IF(B40="NONCI",AND(L40=0,M40=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O40" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L40)),NOT(ISBLANK(M40))),1,"")</f>
         <v>1</v>
       </c>
@@ -4373,13 +4862,13 @@
         <v>39</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E41" s="1" t="n">
         <v>0</v>
@@ -4399,7 +4888,7 @@
       <c r="J41" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K41" s="2" t="b">
+      <c r="K41" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4409,7 +4898,11 @@
       <c r="M41" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N41" s="1" t="n">
+      <c r="N41" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L41),ISBLANK(M41)),"",IF(B41="ADD",AND(L41=1,M41=0),IF(B41="REMOVE",AND(L41=0,M41=1),IF(B41="NONCI",AND(L41=0,M41=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O41" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L41)),NOT(ISBLANK(M41))),1,"")</f>
         <v>1</v>
       </c>
@@ -4419,13 +4912,13 @@
         <v>40</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E42" s="1" t="n">
         <v>0</v>
@@ -4445,7 +4938,7 @@
       <c r="J42" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K42" s="2" t="b">
+      <c r="K42" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4455,7 +4948,11 @@
       <c r="M42" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N42" s="1" t="n">
+      <c r="N42" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L42),ISBLANK(M42)),"",IF(B42="ADD",AND(L42=1,M42=0),IF(B42="REMOVE",AND(L42=0,M42=1),IF(B42="NONCI",AND(L42=0,M42=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O42" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L42)),NOT(ISBLANK(M42))),1,"")</f>
         <v>1</v>
       </c>
@@ -4465,13 +4962,13 @@
         <v>41</v>
       </c>
       <c r="B43" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C43" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C43" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="D43" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E43" s="1" t="n">
         <v>0</v>
@@ -4491,7 +4988,7 @@
       <c r="J43" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K43" s="2" t="b">
+      <c r="K43" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4501,7 +4998,11 @@
       <c r="M43" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N43" s="1" t="n">
+      <c r="N43" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L43),ISBLANK(M43)),"",IF(B43="ADD",AND(L43=1,M43=0),IF(B43="REMOVE",AND(L43=0,M43=1),IF(B43="NONCI",AND(L43=0,M43=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O43" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L43)),NOT(ISBLANK(M43))),1,"")</f>
         <v>1</v>
       </c>
@@ -4511,13 +5012,13 @@
         <v>42</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E44" s="1" t="n">
         <v>0</v>
@@ -4537,7 +5038,7 @@
       <c r="J44" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K44" s="2" t="b">
+      <c r="K44" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4547,7 +5048,11 @@
       <c r="M44" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N44" s="1" t="n">
+      <c r="N44" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L44),ISBLANK(M44)),"",IF(B44="ADD",AND(L44=1,M44=0),IF(B44="REMOVE",AND(L44=0,M44=1),IF(B44="NONCI",AND(L44=0,M44=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O44" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L44)),NOT(ISBLANK(M44))),1,"")</f>
         <v>1</v>
       </c>
@@ -4557,14 +5062,14 @@
         <v>43</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C45" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D45" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="E45" s="1" t="n">
         <v>0</v>
       </c>
@@ -4583,7 +5088,7 @@
       <c r="J45" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K45" s="2" t="b">
+      <c r="K45" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4593,7 +5098,11 @@
       <c r="M45" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N45" s="1" t="n">
+      <c r="N45" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L45),ISBLANK(M45)),"",IF(B45="ADD",AND(L45=1,M45=0),IF(B45="REMOVE",AND(L45=0,M45=1),IF(B45="NONCI",AND(L45=0,M45=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O45" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L45)),NOT(ISBLANK(M45))),1,"")</f>
         <v>1</v>
       </c>
@@ -4603,13 +5112,13 @@
         <v>44</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E46" s="1" t="n">
         <v>0</v>
@@ -4629,7 +5138,7 @@
       <c r="J46" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K46" s="2" t="b">
+      <c r="K46" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4639,7 +5148,11 @@
       <c r="M46" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N46" s="1" t="n">
+      <c r="N46" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L46),ISBLANK(M46)),"",IF(B46="ADD",AND(L46=1,M46=0),IF(B46="REMOVE",AND(L46=0,M46=1),IF(B46="NONCI",AND(L46=0,M46=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O46" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L46)),NOT(ISBLANK(M46))),1,"")</f>
         <v>1</v>
       </c>
@@ -4649,13 +5162,13 @@
         <v>45</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E47" s="1" t="n">
         <v>0</v>
@@ -4675,7 +5188,7 @@
       <c r="J47" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K47" s="2" t="b">
+      <c r="K47" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4685,7 +5198,11 @@
       <c r="M47" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N47" s="1" t="n">
+      <c r="N47" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L47),ISBLANK(M47)),"",IF(B47="ADD",AND(L47=1,M47=0),IF(B47="REMOVE",AND(L47=0,M47=1),IF(B47="NONCI",AND(L47=0,M47=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O47" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L47)),NOT(ISBLANK(M47))),1,"")</f>
         <v>1</v>
       </c>
@@ -4695,13 +5212,13 @@
         <v>46</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E48" s="1" t="n">
         <v>0</v>
@@ -4721,7 +5238,7 @@
       <c r="J48" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K48" s="2" t="b">
+      <c r="K48" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4731,7 +5248,11 @@
       <c r="M48" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N48" s="1" t="n">
+      <c r="N48" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L48),ISBLANK(M48)),"",IF(B48="ADD",AND(L48=1,M48=0),IF(B48="REMOVE",AND(L48=0,M48=1),IF(B48="NONCI",AND(L48=0,M48=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O48" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L48)),NOT(ISBLANK(M48))),1,"")</f>
         <v>1</v>
       </c>
@@ -4741,13 +5262,13 @@
         <v>47</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E49" s="1" t="n">
         <v>0</v>
@@ -4767,7 +5288,7 @@
       <c r="J49" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K49" s="2" t="b">
+      <c r="K49" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4777,7 +5298,11 @@
       <c r="M49" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N49" s="1" t="n">
+      <c r="N49" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L49),ISBLANK(M49)),"",IF(B49="ADD",AND(L49=1,M49=0),IF(B49="REMOVE",AND(L49=0,M49=1),IF(B49="NONCI",AND(L49=0,M49=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O49" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L49)),NOT(ISBLANK(M49))),1,"")</f>
         <v>1</v>
       </c>
@@ -4787,13 +5312,13 @@
         <v>48</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E50" s="1" t="n">
         <v>0</v>
@@ -4813,7 +5338,7 @@
       <c r="J50" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K50" s="2" t="b">
+      <c r="K50" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4823,7 +5348,11 @@
       <c r="M50" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N50" s="1" t="n">
+      <c r="N50" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L50),ISBLANK(M50)),"",IF(B50="ADD",AND(L50=1,M50=0),IF(B50="REMOVE",AND(L50=0,M50=1),IF(B50="NONCI",AND(L50=0,M50=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O50" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L50)),NOT(ISBLANK(M50))),1,"")</f>
         <v>1</v>
       </c>
@@ -4833,13 +5362,13 @@
         <v>49</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E51" s="1" t="n">
         <v>0</v>
@@ -4859,7 +5388,7 @@
       <c r="J51" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K51" s="2" t="b">
+      <c r="K51" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4869,7 +5398,11 @@
       <c r="M51" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N51" s="1" t="n">
+      <c r="N51" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L51),ISBLANK(M51)),"",IF(B51="ADD",AND(L51=1,M51=0),IF(B51="REMOVE",AND(L51=0,M51=1),IF(B51="NONCI",AND(L51=0,M51=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O51" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L51)),NOT(ISBLANK(M51))),1,"")</f>
         <v>1</v>
       </c>
@@ -4879,13 +5412,13 @@
         <v>50</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E52" s="1" t="n">
         <v>0</v>
@@ -4905,7 +5438,7 @@
       <c r="J52" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K52" s="2" t="b">
+      <c r="K52" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4915,7 +5448,11 @@
       <c r="M52" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N52" s="1" t="n">
+      <c r="N52" s="3" t="b">
+        <f aca="false">IF(OR(ISBLANK(L52),ISBLANK(M52)),"",IF(B52="ADD",AND(L52=1,M52=0),IF(B52="REMOVE",AND(L52=0,M52=1),IF(B52="NONCI",AND(L52=0,M52=0),"" ))))</f>
+        <v>1</v>
+      </c>
+      <c r="O52" s="1" t="n">
         <f aca="false">IF(AND(NOT(ISBLANK(L52)),NOT(ISBLANK(M52))),1,"")</f>
         <v>1</v>
       </c>

</xml_diff>